<commit_message>
add africa and CIS from hatayama10
</commit_message>
<xml_diff>
--- a/lifetime_input/input/lifetime_table.xlsx
+++ b/lifetime_input/input/lifetime_table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bennetwe\Documents\Code\posted\lifetime_input_output\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bennetwe\Documents\Code\posted\lifetime_input\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752A0895-665A-4A68-B7C5-21246C2CA3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5256788-5C51-448C-ABC7-89C49C7D0526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="36">
   <si>
     <t>1950-1969</t>
   </si>
@@ -133,6 +133,15 @@
   </si>
   <si>
     <t>source_detail</t>
+  </si>
+  <si>
+    <t>CIS</t>
+  </si>
+  <si>
+    <t>Hatayama10</t>
+  </si>
+  <si>
+    <t>Afrika</t>
   </si>
 </sst>
 </file>
@@ -1051,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E207A79-48E6-4E24-B73D-E7824509D926}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1549,6 +1558,52 @@
         <v>19</v>
       </c>
     </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22">
+        <v>60</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23">
+        <v>60</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H23" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>